<commit_message>
Atualização dos painéis em 30/09/2026 16:15 por Danielle Guimarães
</commit_message>
<xml_diff>
--- a/dados/iicp-iipr.xlsx
+++ b/dados/iicp-iipr.xlsx
@@ -14471,13 +14471,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E24CD1F-A37E-44A4-A600-18511F6E76CC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5A9EDF4-824C-4705-A255-7611CD6D732B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C210BC4-D9E1-4473-B7F9-E41BF11FA396}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98C5E847-B925-4FF9-946B-81BF3081FFD6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4A07DA4-6B60-4449-A561-7F6A7312924A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{625A4E5A-4F6E-4B25-BA13-B81AF81E65C5}"/>
 </file>
</xml_diff>

<commit_message>
Atualização dos painéis em 01/10/2026 16:12 por Danielle Guimarães
</commit_message>
<xml_diff>
--- a/dados/iicp-iipr.xlsx
+++ b/dados/iicp-iipr.xlsx
@@ -473,7 +473,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dados até 08/2026. Arquivo gerado em 30/09/2026.</t>
+          <t>Dados até 08/2026. Arquivo gerado em 01/10/2026.</t>
         </is>
       </c>
     </row>
@@ -14471,13 +14471,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5A9EDF4-824C-4705-A255-7611CD6D732B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4314A467-5FD7-46FB-82D5-5197FC400A11}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98C5E847-B925-4FF9-946B-81BF3081FFD6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84ADB3AD-A2CB-489F-9BDF-D51111FDA793}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{625A4E5A-4F6E-4B25-BA13-B81AF81E65C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79DAF1D6-E2D5-4AFA-8882-ED06D614610B}"/>
 </file>
</xml_diff>

<commit_message>
Atualização dos painéis em 29/10/2026 09:57 por Ruy Silveira Neto
</commit_message>
<xml_diff>
--- a/dados/iicp-iipr.xlsx
+++ b/dados/iicp-iipr.xlsx
@@ -473,7 +473,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dados até 08/2026. Arquivo gerado em 01/10/2026.</t>
+          <t>Dados até 09/2026. Arquivo gerado em 29/10/2026.</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3764,7 +3764,7 @@
         <v>167.1165</v>
       </c>
       <c r="C188" s="5" t="n">
-        <v>285.6401</v>
+        <v>285.6264</v>
       </c>
       <c r="D188" s="5" t="n">
         <v>241.9944</v>
@@ -3798,7 +3798,7 @@
         <v>166.4554</v>
       </c>
       <c r="C190" s="5" t="n">
-        <v>283.7126</v>
+        <v>283.6944</v>
       </c>
       <c r="D190" s="5" t="n">
         <v>242.8885</v>
@@ -3815,7 +3815,7 @@
         <v>164.5638</v>
       </c>
       <c r="C191" s="5" t="n">
-        <v>277.9811</v>
+        <v>277.9221</v>
       </c>
       <c r="D191" s="5" t="n">
         <v>243.1071</v>
@@ -3832,7 +3832,7 @@
         <v>163.4447</v>
       </c>
       <c r="C192" s="5" t="n">
-        <v>277.0358</v>
+        <v>276.954</v>
       </c>
       <c r="D192" s="5" t="n">
         <v>243.5447</v>
@@ -3849,7 +3849,7 @@
         <v>163.6349</v>
       </c>
       <c r="C193" s="5" t="n">
-        <v>277.6028</v>
+        <v>277.4302</v>
       </c>
       <c r="D193" s="5" t="n">
         <v>244.3484</v>
@@ -3866,7 +3866,7 @@
         <v>164.4683</v>
       </c>
       <c r="C194" s="5" t="n">
-        <v>272.8115</v>
+        <v>272.5708</v>
       </c>
       <c r="D194" s="5" t="n">
         <v>245.1547</v>
@@ -3883,7 +3883,7 @@
         <v>162.7957</v>
       </c>
       <c r="C195" s="5" t="n">
-        <v>264.853</v>
+        <v>264.6165</v>
       </c>
       <c r="D195" s="5" t="n">
         <v>246.8708</v>
@@ -3900,7 +3900,7 @@
         <v>170.6347</v>
       </c>
       <c r="C196" s="5" t="n">
-        <v>269.5575</v>
+        <v>269.3576</v>
       </c>
       <c r="D196" s="5" t="n">
         <v>249.0433</v>
@@ -3917,7 +3917,7 @@
         <v>173.2876</v>
       </c>
       <c r="C197" s="5" t="n">
-        <v>271.7525</v>
+        <v>271.6525</v>
       </c>
       <c r="D197" s="5" t="n">
         <v>250.7119</v>
@@ -3934,7 +3934,7 @@
         <v>173.3516</v>
       </c>
       <c r="C198" s="5" t="n">
-        <v>266.3755</v>
+        <v>266.3301</v>
       </c>
       <c r="D198" s="5" t="n">
         <v>252.166</v>
@@ -3951,7 +3951,7 @@
         <v>171.2099</v>
       </c>
       <c r="C199" s="5" t="n">
-        <v>266.8898</v>
+        <v>266.858</v>
       </c>
       <c r="D199" s="5" t="n">
         <v>252.5694</v>
@@ -3968,7 +3968,7 @@
         <v>169.1846</v>
       </c>
       <c r="C200" s="5" t="n">
-        <v>284.1998</v>
+        <v>284.1862</v>
       </c>
       <c r="D200" s="5" t="n">
         <v>252.7462</v>
@@ -3985,13 +3985,30 @@
         <v>169.5953</v>
       </c>
       <c r="C201" s="5" t="n">
-        <v>299.9917</v>
+        <v>300.0054</v>
       </c>
       <c r="D201" s="5" t="n">
         <v>251.9375</v>
       </c>
       <c r="E201" s="5" t="n">
         <v>317.1313</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B202" s="5" t="n">
+        <v>172.036</v>
+      </c>
+      <c r="C202" s="5" t="n">
+        <v>322.637</v>
+      </c>
+      <c r="D202" s="5" t="n">
+        <v>254.0033</v>
+      </c>
+      <c r="E202" s="5" t="n">
+        <v>319.7635</v>
       </c>
     </row>
   </sheetData>
@@ -4005,7 +4022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7208,7 +7225,7 @@
         <v>-0.009256</v>
       </c>
       <c r="C188" s="6" t="n">
-        <v>0.00827</v>
+        <v>0.008222</v>
       </c>
       <c r="D188" s="6" t="n">
         <v>0.0026</v>
@@ -7225,7 +7242,7 @@
         <v>-0.001616</v>
       </c>
       <c r="C189" s="6" t="n">
-        <v>0.009427</v>
+        <v>0.009475000000000001</v>
       </c>
       <c r="D189" s="6" t="n">
         <v>-0.0011</v>
@@ -7242,7 +7259,7 @@
         <v>-0.002344</v>
       </c>
       <c r="C190" s="6" t="n">
-        <v>-0.016024</v>
+        <v>-0.016087</v>
       </c>
       <c r="D190" s="6" t="n">
         <v>0.0048</v>
@@ -7259,7 +7276,7 @@
         <v>-0.011364</v>
       </c>
       <c r="C191" s="6" t="n">
-        <v>-0.020202</v>
+        <v>-0.020347</v>
       </c>
       <c r="D191" s="6" t="n">
         <v>0.0009</v>
@@ -7276,7 +7293,7 @@
         <v>-0.0068</v>
       </c>
       <c r="C192" s="6" t="n">
-        <v>-0.003401</v>
+        <v>-0.003483</v>
       </c>
       <c r="D192" s="6" t="n">
         <v>0.0018</v>
@@ -7293,7 +7310,7 @@
         <v>0.001164</v>
       </c>
       <c r="C193" s="6" t="n">
-        <v>0.002047</v>
+        <v>0.001719</v>
       </c>
       <c r="D193" s="6" t="n">
         <v>0.0033</v>
@@ -7310,7 +7327,7 @@
         <v>0.005093</v>
       </c>
       <c r="C194" s="6" t="n">
-        <v>-0.01726</v>
+        <v>-0.017516</v>
       </c>
       <c r="D194" s="6" t="n">
         <v>0.0033</v>
@@ -7327,7 +7344,7 @@
         <v>-0.01017</v>
       </c>
       <c r="C195" s="6" t="n">
-        <v>-0.029172</v>
+        <v>-0.029182</v>
       </c>
       <c r="D195" s="6" t="n">
         <v>0.007</v>
@@ -7344,7 +7361,7 @@
         <v>0.048153</v>
       </c>
       <c r="C196" s="6" t="n">
-        <v>0.017763</v>
+        <v>0.017917</v>
       </c>
       <c r="D196" s="6" t="n">
         <v>0.008800000000000001</v>
@@ -7361,7 +7378,7 @@
         <v>0.015547</v>
       </c>
       <c r="C197" s="6" t="n">
-        <v>0.008142999999999999</v>
+        <v>0.00852</v>
       </c>
       <c r="D197" s="6" t="n">
         <v>0.0067</v>
@@ -7378,7 +7395,7 @@
         <v>0.00037</v>
       </c>
       <c r="C198" s="6" t="n">
-        <v>-0.019786</v>
+        <v>-0.019593</v>
       </c>
       <c r="D198" s="6" t="n">
         <v>0.0058</v>
@@ -7395,7 +7412,7 @@
         <v>-0.012354</v>
       </c>
       <c r="C199" s="6" t="n">
-        <v>0.001931</v>
+        <v>0.001982</v>
       </c>
       <c r="D199" s="6" t="n">
         <v>0.0016</v>
@@ -7412,7 +7429,7 @@
         <v>-0.011829</v>
       </c>
       <c r="C200" s="6" t="n">
-        <v>0.064858</v>
+        <v>0.06493400000000001</v>
       </c>
       <c r="D200" s="6" t="n">
         <v>0.0007</v>
@@ -7429,13 +7446,30 @@
         <v>0.002427</v>
       </c>
       <c r="C201" s="6" t="n">
-        <v>0.055566</v>
+        <v>0.055665</v>
       </c>
       <c r="D201" s="6" t="n">
         <v>-0.0032</v>
       </c>
       <c r="E201" s="6" t="n">
         <v>-0.0034</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B202" s="6" t="n">
+        <v>0.014392</v>
+      </c>
+      <c r="C202" s="6" t="n">
+        <v>0.075437</v>
+      </c>
+      <c r="D202" s="6" t="n">
+        <v>0.008200000000000001</v>
+      </c>
+      <c r="E202" s="6" t="n">
+        <v>0.0083</v>
       </c>
     </row>
   </sheetData>
@@ -7449,7 +7483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10582,7 +10616,7 @@
         <v>0.010991</v>
       </c>
       <c r="C188" s="6" t="n">
-        <v>-0.103107</v>
+        <v>-0.10315</v>
       </c>
       <c r="D188" s="6" t="n">
         <v>0.0326</v>
@@ -10616,7 +10650,7 @@
         <v>0.006991</v>
       </c>
       <c r="C190" s="6" t="n">
-        <v>-0.109159</v>
+        <v>-0.109216</v>
       </c>
       <c r="D190" s="6" t="n">
         <v>0.0364</v>
@@ -10633,7 +10667,7 @@
         <v>-0.004452</v>
       </c>
       <c r="C191" s="6" t="n">
-        <v>-0.127156</v>
+        <v>-0.127341</v>
       </c>
       <c r="D191" s="6" t="n">
         <v>0.0373</v>
@@ -10650,7 +10684,7 @@
         <v>-0.011223</v>
       </c>
       <c r="C192" s="6" t="n">
-        <v>-0.130124</v>
+        <v>-0.130381</v>
       </c>
       <c r="D192" s="6" t="n">
         <v>0.0393</v>
@@ -10667,7 +10701,7 @@
         <v>-0.010072</v>
       </c>
       <c r="C193" s="6" t="n">
-        <v>-0.128343</v>
+        <v>-0.128885</v>
       </c>
       <c r="D193" s="6" t="n">
         <v>0.0426</v>
@@ -10684,7 +10718,7 @@
         <v>0.005093</v>
       </c>
       <c r="C194" s="6" t="n">
-        <v>-0.01726</v>
+        <v>-0.017516</v>
       </c>
       <c r="D194" s="6" t="n">
         <v>0.0033</v>
@@ -10701,7 +10735,7 @@
         <v>-0.005128</v>
       </c>
       <c r="C195" s="6" t="n">
-        <v>-0.045928</v>
+        <v>-0.046187</v>
       </c>
       <c r="D195" s="6" t="n">
         <v>0.0103</v>
@@ -10718,7 +10752,7 @@
         <v>0.042777</v>
       </c>
       <c r="C196" s="6" t="n">
-        <v>-0.028982</v>
+        <v>-0.029098</v>
       </c>
       <c r="D196" s="6" t="n">
         <v>0.0192</v>
@@ -10735,7 +10769,7 @@
         <v>0.058989</v>
       </c>
       <c r="C197" s="6" t="n">
-        <v>-0.021075</v>
+        <v>-0.020826</v>
       </c>
       <c r="D197" s="6" t="n">
         <v>0.026</v>
@@ -10752,7 +10786,7 @@
         <v>0.059381</v>
       </c>
       <c r="C198" s="6" t="n">
-        <v>-0.040444</v>
+        <v>-0.04001</v>
       </c>
       <c r="D198" s="6" t="n">
         <v>0.032</v>
@@ -10769,7 +10803,7 @@
         <v>0.046293</v>
       </c>
       <c r="C199" s="6" t="n">
-        <v>-0.038591</v>
+        <v>-0.038108</v>
       </c>
       <c r="D199" s="6" t="n">
         <v>0.0336</v>
@@ -10786,7 +10820,7 @@
         <v>0.033916</v>
       </c>
       <c r="C200" s="6" t="n">
-        <v>0.023764</v>
+        <v>0.024352</v>
       </c>
       <c r="D200" s="6" t="n">
         <v>0.0344</v>
@@ -10803,13 +10837,30 @@
         <v>0.036425</v>
       </c>
       <c r="C201" s="6" t="n">
-        <v>0.080651</v>
+        <v>0.081372</v>
       </c>
       <c r="D201" s="6" t="n">
         <v>0.0311</v>
       </c>
       <c r="E201" s="6" t="n">
         <v>0.0352</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B202" s="6" t="n">
+        <v>0.051341</v>
+      </c>
+      <c r="C202" s="6" t="n">
+        <v>0.162948</v>
+      </c>
+      <c r="D202" s="6" t="n">
+        <v>0.0395</v>
+      </c>
+      <c r="E202" s="6" t="n">
+        <v>0.0437</v>
       </c>
     </row>
   </sheetData>
@@ -10823,7 +10874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13960,7 +14011,7 @@
         <v>0.015459</v>
       </c>
       <c r="C188" s="6" t="n">
-        <v>-0.099513</v>
+        <v>-0.09955600000000001</v>
       </c>
       <c r="D188" s="6" t="n">
         <v>0.0523</v>
@@ -13994,7 +14045,7 @@
         <v>0.006776</v>
       </c>
       <c r="C190" s="6" t="n">
-        <v>-0.114358</v>
+        <v>-0.114415</v>
       </c>
       <c r="D190" s="6" t="n">
         <v>0.0517</v>
@@ -14011,7 +14062,7 @@
         <v>-0.003939</v>
       </c>
       <c r="C191" s="6" t="n">
-        <v>-0.143743</v>
+        <v>-0.143925</v>
       </c>
       <c r="D191" s="6" t="n">
         <v>0.0468</v>
@@ -14028,7 +14079,7 @@
         <v>-0.005875</v>
       </c>
       <c r="C192" s="6" t="n">
-        <v>-0.1561</v>
+        <v>-0.156349</v>
       </c>
       <c r="D192" s="6" t="n">
         <v>0.0446</v>
@@ -14045,7 +14096,7 @@
         <v>-0.010072</v>
       </c>
       <c r="C193" s="6" t="n">
-        <v>-0.128343</v>
+        <v>-0.128885</v>
       </c>
       <c r="D193" s="6" t="n">
         <v>0.0426</v>
@@ -14062,7 +14113,7 @@
         <v>-0.029472</v>
       </c>
       <c r="C194" s="6" t="n">
-        <v>-0.140404</v>
+        <v>-0.141163</v>
       </c>
       <c r="D194" s="6" t="n">
         <v>0.0444</v>
@@ -14079,7 +14130,7 @@
         <v>-0.044371</v>
       </c>
       <c r="C195" s="6" t="n">
-        <v>-0.136089</v>
+        <v>-0.13686</v>
       </c>
       <c r="D195" s="6" t="n">
         <v>0.0381</v>
@@ -14096,7 +14147,7 @@
         <v>0.014871</v>
       </c>
       <c r="C196" s="6" t="n">
-        <v>-0.119091</v>
+        <v>-0.119744</v>
       </c>
       <c r="D196" s="6" t="n">
         <v>0.0414</v>
@@ -14113,7 +14164,7 @@
         <v>0.023721</v>
       </c>
       <c r="C197" s="6" t="n">
-        <v>-0.091876</v>
+        <v>-0.09221</v>
       </c>
       <c r="D197" s="6" t="n">
         <v>0.0439</v>
@@ -14130,7 +14181,7 @@
         <v>0.031146</v>
       </c>
       <c r="C198" s="6" t="n">
-        <v>-0.076366</v>
+        <v>-0.07652299999999999</v>
       </c>
       <c r="D198" s="6" t="n">
         <v>0.0472</v>
@@ -14147,7 +14198,7 @@
         <v>0.015012</v>
       </c>
       <c r="C199" s="6" t="n">
-        <v>-0.057916</v>
+        <v>-0.058028</v>
       </c>
       <c r="D199" s="6" t="n">
         <v>0.0464</v>
@@ -14181,13 +14232,30 @@
         <v>0.016475</v>
       </c>
       <c r="C201" s="6" t="n">
-        <v>0.040436</v>
+        <v>0.040483</v>
       </c>
       <c r="D201" s="6" t="n">
         <v>0.0422</v>
       </c>
       <c r="E201" s="6" t="n">
         <v>0.0353</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B202" s="6" t="n">
+        <v>0.033526</v>
+      </c>
+      <c r="C202" s="6" t="n">
+        <v>0.13727</v>
+      </c>
+      <c r="D202" s="6" t="n">
+        <v>0.0458</v>
+      </c>
+      <c r="E202" s="6" t="n">
+        <v>0.0466</v>
       </c>
     </row>
   </sheetData>
@@ -14471,13 +14539,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4314A467-5FD7-46FB-82D5-5197FC400A11}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E2AA955-ECF9-4BC9-BA73-61A2F4525B6E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84ADB3AD-A2CB-489F-9BDF-D51111FDA793}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C47E964-FBF1-4392-A7E1-9250579E75C4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79DAF1D6-E2D5-4AFA-8882-ED06D614610B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75C195F9-D12D-4A40-92F0-8E7934726C54}"/>
 </file>
</xml_diff>